<commit_message>
Shorten baseline benchmark evidence paths for Windows
Remove the redundant archive-name directory and update source paths in the merged workbook, JSON and CSVs. Preserve original evidence bytes and all selected benchmark values.
</commit_message>
<xml_diff>
--- a/docs/benchmarks/MFCC_Benchmark_Summary.xlsx
+++ b/docs/benchmarks/MFCC_Benchmark_Summary.xlsx
@@ -881,7 +881,7 @@
       </c>
       <c r="P13" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/synthesis/new_n512_lanes1/utilization.rpt</t>
+          <t>evidence/baseline/raw_reports/synthesis/new_n512_lanes1/utilization.rpt</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="J2" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="J3" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3723,7 +3723,7 @@
       </c>
       <c r="J4" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3761,7 +3761,7 @@
       </c>
       <c r="J5" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="J6" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="J7" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3875,7 +3875,7 @@
       </c>
       <c r="J8" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3913,7 +3913,7 @@
       </c>
       <c r="J9" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3951,7 @@
       </c>
       <c r="J10" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3989,7 @@
       </c>
       <c r="J11" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -4027,7 +4027,7 @@
       </c>
       <c r="J12" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="L2" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/runtime_fft_speed_50MHz.csv</t>
+          <t>evidence/baseline/runtime_fft_speed_50MHz.csv</t>
         </is>
       </c>
       <c r="M2" s="0" t="inlineStr">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="L3" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/runtime_fft_speed_50MHz.csv</t>
+          <t>evidence/baseline/runtime_fft_speed_50MHz.csv</t>
         </is>
       </c>
       <c r="M3" s="0" t="inlineStr">
@@ -4713,7 +4713,7 @@
       </c>
       <c r="L4" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/runtime_fft_speed_50MHz.csv</t>
+          <t>evidence/baseline/runtime_fft_speed_50MHz.csv</t>
         </is>
       </c>
       <c r="M4" s="0" t="inlineStr">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="L5" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/runtime_fft_speed_50MHz.csv</t>
+          <t>evidence/baseline/runtime_fft_speed_50MHz.csv</t>
         </is>
       </c>
       <c r="M5" s="0" t="inlineStr">
@@ -4807,7 +4807,7 @@
       </c>
       <c r="L6" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/runtime_fft_speed_50MHz.csv</t>
+          <t>evidence/baseline/runtime_fft_speed_50MHz.csv</t>
         </is>
       </c>
       <c r="M6" s="0" t="inlineStr">
@@ -4854,7 +4854,7 @@
       </c>
       <c r="L7" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/runtime_fft_speed_50MHz.csv</t>
+          <t>evidence/baseline/runtime_fft_speed_50MHz.csv</t>
         </is>
       </c>
       <c r="M7" s="0" t="inlineStr">
@@ -4901,7 +4901,7 @@
       </c>
       <c r="L8" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/runtime_fft_speed_50MHz.csv</t>
+          <t>evidence/baseline/runtime_fft_speed_50MHz.csv</t>
         </is>
       </c>
       <c r="M8" s="0" t="inlineStr">
@@ -4948,7 +4948,7 @@
       </c>
       <c r="L9" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/runtime_fft_speed_50MHz.csv</t>
+          <t>evidence/baseline/runtime_fft_speed_50MHz.csv</t>
         </is>
       </c>
       <c r="M9" s="0" t="inlineStr">
@@ -6344,7 +6344,7 @@
       </c>
       <c r="K2" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6383,7 +6383,7 @@
       </c>
       <c r="K3" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6422,7 +6422,7 @@
       </c>
       <c r="K4" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6461,7 +6461,7 @@
       </c>
       <c r="K5" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6500,7 +6500,7 @@
       </c>
       <c r="K6" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6539,7 +6539,7 @@
       </c>
       <c r="K7" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6578,7 +6578,7 @@
       </c>
       <c r="K8" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6617,7 +6617,7 @@
       </c>
       <c r="K9" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6656,7 +6656,7 @@
       </c>
       <c r="K10" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6695,7 +6695,7 @@
       </c>
       <c r="K11" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>
@@ -6734,7 +6734,7 @@
       </c>
       <c r="K12" s="0" t="inlineStr">
         <is>
-          <t>evidence/baseline/KV260_working_mfcc_fft_bram_tested_20261022/raw_reports/mfcc_integration.json</t>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace MatrixDCT BRAM storage with registers and LUT ROM
Preserve the public interface and numerical behavior, with separate operand,
product and accumulation stages. Validate against the prior RTL and an
independent integer model, plus complete-MFCC regression configurations.

Refresh benchmark summaries and mark replacement hardware metrics pending.
</commit_message>
<xml_diff>
--- a/docs/benchmarks/MFCC_Benchmark_Summary.xlsx
+++ b/docs/benchmarks/MFCC_Benchmark_Summary.xlsx
@@ -673,33 +673,49 @@
       <c r="E10" s="2">
         <v>64</v>
       </c>
-      <c r="F10" s="2">
-        <v>647</v>
-      </c>
-      <c r="G10" s="3">
-        <v>0.55</v>
-      </c>
-      <c r="H10" s="2">
-        <v>1098</v>
-      </c>
-      <c r="I10" s="3">
-        <v>0.47</v>
-      </c>
-      <c r="J10" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="K10" s="3">
-        <v>1.74</v>
-      </c>
-      <c r="L10" s="2">
-        <v>1</v>
-      </c>
-      <c r="M10" s="3">
-        <v>0.08</v>
+      <c r="F10" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G10" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H10" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I10" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J10" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K10" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L10" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M10" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="N10" s="0" t="inlineStr">
         <is>
-          <t>OOC post-route; hierarchy inclusive</t>
+          <t>Register/LUT RTL; hardware reimplementation pending</t>
         </is>
       </c>
       <c r="O10" s="3">
@@ -707,7 +723,7 @@
       </c>
       <c r="P10" s="0" t="inlineStr">
         <is>
-          <t>recursive_skewdct_N1024_20261026/raw_reports/matrixdct_50MHz/utilization_hierarchical_post_route.rpt</t>
+          <t>matrix_register_20261026/verified_results.json</t>
         </is>
       </c>
     </row>
@@ -905,33 +921,49 @@
       <c r="E14" s="2">
         <v>64</v>
       </c>
-      <c r="F14" s="2">
-        <v>30188</v>
-      </c>
-      <c r="G14" s="3">
-        <v>25.78</v>
-      </c>
-      <c r="H14" s="2">
-        <v>41987</v>
-      </c>
-      <c r="I14" s="3">
-        <v>17.92</v>
-      </c>
-      <c r="J14" s="3">
-        <v>9.0</v>
-      </c>
-      <c r="K14" s="3">
-        <v>6.25</v>
-      </c>
-      <c r="L14" s="2">
-        <v>19</v>
-      </c>
-      <c r="M14" s="3">
-        <v>1.52</v>
+      <c r="F14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M14" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="N14" s="0" t="inlineStr">
         <is>
-          <t>OOC post-route; hierarchy inclusive</t>
+          <t>Register/LUT RTL; hardware reimplementation pending</t>
         </is>
       </c>
       <c r="O14" s="3">
@@ -939,7 +971,7 @@
       </c>
       <c r="P14" s="0" t="inlineStr">
         <is>
-          <t>recursive_skewdct_N1024_20261026/raw_reports/matrixdct_50MHz/utilization_hierarchical_post_route.rpt</t>
+          <t>matrix_register_20261026/verified_results.json</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2466,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2641,8 +2673,30 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="0" t="inlineStr">
+        <is>
+          <t>MatrixDCT register/LUT replacement</t>
+        </is>
+      </c>
+      <c r="B10" s="0" t="inlineStr">
+        <is>
+          <t>Six unit cases; twenty MFCC configurations</t>
+        </is>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Simulation passes; new physical resource/timing mapping pending</t>
+        </is>
+      </c>
+      <c r="D10" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_20261026/README.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:D10"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -2916,7 +2970,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2938,149 +2992,161 @@
     <row r="2">
       <c r="A2" s="0" t="inlineStr">
         <is>
-          <t>Selection rule</t>
+          <t>MatrixDCT storage replacement</t>
         </is>
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>Keep the latest valid value per test project and configuration. Architecture/pipeline/version names are not separate test projects.</t>
+          <t>Current MatrixDCT uses register/LUT storage. Its new resource and timing fields are pending, not copied from the obsolete BRAM implementation. Latest verified N1024 batch: 43622 cycles. Original hardware reports remain historical evidence.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>Configuration key</t>
+          <t>Selection rule</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>Project, backend under comparison, N, frequency, output lanes, frame count and stall condition identify a case. Inclusive hierarchy scope is retained.</t>
+          <t>Keep the latest valid value per test project and configuration. Architecture/pipeline/version names are not separate test projects.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>Partial updates</t>
+          <t>Configuration key</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Refresh metrics separately: a 150 MHz resource update does not invent new 50/100 MHz resources. Unchanged metrics use the latest available reports. Runtime cycle counts use the latest matching regression and are converted by frequency.</t>
+          <t>Project, backend under comparison, N, frequency, output lanes, frame count and stall condition identify a case. Inclusive hierarchy scope is retained.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Partial updates</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>Source paths in tables and JSON are relative to docs/benchmarks/. Per-metric source columns identify the original evidence; different metric groups can come from different packages.</t>
+          <t>Refresh metrics separately: a 150 MHz resource update does not invent new 50/100 MHz resources. Unchanged metrics use the latest available reports. Runtime cycle counts use the latest matching regression and are converted by frequency.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>Resource priority</t>
+          <t>Sources</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>LUT, FF, BRAM and DSP appear first. DCT/C64/SkewDCT8 hierarchy rows are already included in parent totals.</t>
+          <t>Source paths in tables and JSON are relative to docs/benchmarks/. Per-metric source columns identify the original evidence; different metric groups can come from different packages.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>BRAM unit</t>
+          <t>Resource priority</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>One BRAM tile is a 36 Kb equivalent; each RAMB18 counts as 0.5 tile.</t>
+          <t>LUT, FF, BRAM and DSP appear first. DCT/C64/SkewDCT8 hierarchy rows are already included in parent totals.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>FFT evidence</t>
+          <t>BRAM unit</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>XFFT resource reports use fixed-size cores and a 10 ns synthesis clock; custom FFT resources use a shared runtime core after routing at 20 ns. The 64..2048 XFFT latency numbers use runtime_2048. These attributes remain source metadata, not version-specific result rows.</t>
+          <t>One BRAM tile is a 36 Kb equivalent; each RAMB18 counts as 0.5 tile.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>FFT 16-point counting</t>
+          <t>FFT evidence</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>Latest reported custom complete-frame latency is 82 cycles; its accompanying regression records 83. The primary table retains the latest reported value and marks this counting discrepancy.</t>
+          <t>XFFT resource reports use fixed-size cores and a 10 ns synthesis clock; custom FFT resources use a shared runtime core after routing at 20 ns. The 64..2048 XFFT latency numbers use runtime_2048. These attributes remain source metadata, not version-specific result rows.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>FFT first output</t>
+          <t>FFT 16-point counting</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>First-output cycles are taken from the latest package reporting that metric (2026-10-22); complete-frame comparisons are updated by the 2026-10-25 package.</t>
+          <t>Latest reported custom complete-frame latency is 82 cycles; its accompanying regression records 83. The primary table retains the latest reported value and marks this counting discrepancy.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>Timing/accuracy scope</t>
+          <t>FFT first output</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>Times are RTL cycles divided by MHz, not board/PS/DMA measurements. Four-frame averages are not independently measured single-frame latency or steady-state II. MFCC reference errors do not isolate DCT error or recognition accuracy.</t>
+          <t>First-output cycles are taken from the latest package reporting that metric (2026-10-22); complete-frame comparisons are updated by the 2026-10-25 package.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>Timing/accuracy scope</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>Superseded values remain in immutable original reports for traceability, outside primary tables. The explicit paired memory before/after experiment retains both required comparison sides.</t>
+          <t>Times are RTL cycles divided by MHz, not board/PS/DMA measurements. Four-frame averages are not independently measured single-frame latency or steady-state II. MFCC reference errors do not isolate DCT error or recognition accuracy.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="B13" s="0" t="inlineStr">
+        <is>
+          <t>Superseded values remain in immutable original reports for traceability, outside primary tables. The explicit paired memory before/after experiment retains both required comparison sides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="0" t="inlineStr">
+        <is>
           <t>200 MHz status</t>
         </is>
       </c>
-      <c r="B13" s="0" t="inlineStr">
+      <c r="B14" s="0" t="inlineStr">
         <is>
           <t>Not measured for the latest RTL. Frozen-route estimate is approximately -1.409 ns. The old 200 MHz run was interrupted during placement and is not a pass/fail result.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B13"/>
+  <autoFilter ref="A1:B14"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -3481,60 +3547,78 @@
       <c r="F5" s="2">
         <v>50</v>
       </c>
-      <c r="G5" s="2">
-        <v>30188</v>
-      </c>
-      <c r="H5" s="2">
-        <v>41987</v>
-      </c>
-      <c r="I5" s="3">
-        <v>9.0</v>
-      </c>
-      <c r="J5" s="2">
-        <v>19</v>
-      </c>
-      <c r="K5" s="3">
-        <v>8.254</v>
-      </c>
-      <c r="L5" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="M5" s="2">
-        <v>0</v>
-      </c>
-      <c r="N5" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="O5" s="2">
-        <v>0</v>
+      <c r="G5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O5" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
       </c>
       <c r="P5" s="0" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>PENDING_REGISTER_IMPLEMENTATION</t>
         </is>
       </c>
       <c r="Q5" s="2">
-        <v>43687</v>
+        <v>43622</v>
       </c>
       <c r="R5" s="3">
-        <v>873.74</v>
+        <v>872.44</v>
       </c>
       <c r="S5" s="3">
-        <v>218.435</v>
+        <v>218.11</v>
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t>recursive_skewdct_N1024_20261026/raw_reports/matrixdct_50MHz/utilization_hierarchical_post_route.rpt</t>
+          <t>matrix_register_20261026/verified_results.json</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t>recursive_skewdct_N1024_20261026/raw_reports/matrixdct_50MHz/timing_post_route.rpt</t>
+          <t>matrix_register_20261026/verified_results.json</t>
         </is>
       </c>
       <c r="V5" s="0" t="inlineStr">
         <is>
-          <t>c64_pipeline_N1024_150MHz_20261026/results/rtl_precision_performance.json</t>
+          <t>matrix_register_20261026/verified_results.json</t>
         </is>
       </c>
     </row>
@@ -5766,7 +5850,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:W3"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -5781,16 +5865,17 @@
     <col min="10" max="10" width="15" customWidth="1"/>
     <col min="11" max="11" width="15" customWidth="1"/>
     <col min="12" max="12" width="15" customWidth="1"/>
-    <col min="13" max="13" width="15" customWidth="1"/>
+    <col min="13" max="13" width="17" customWidth="1"/>
     <col min="14" max="14" width="15" customWidth="1"/>
     <col min="15" max="15" width="15" customWidth="1"/>
     <col min="16" max="16" width="15" customWidth="1"/>
     <col min="17" max="17" width="15" customWidth="1"/>
-    <col min="18" max="18" width="20" customWidth="1"/>
-    <col min="19" max="19" width="15" customWidth="1"/>
-    <col min="20" max="20" width="65" customWidth="1"/>
+    <col min="18" max="18" width="15" customWidth="1"/>
+    <col min="19" max="19" width="20" customWidth="1"/>
+    <col min="20" max="20" width="15" customWidth="1"/>
     <col min="21" max="21" width="65" customWidth="1"/>
     <col min="22" max="22" width="65" customWidth="1"/>
+    <col min="23" max="23" width="65" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -5856,50 +5941,55 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
+          <t>Hardware status</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>Frames</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Batch cycles</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Batch us</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>MFCC MAE</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>MFCC RMSE</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>MFCC max abs error</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>MFCC SNR dB</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>MFCC resource source</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>DCT resource source</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>Runtime/precision source</t>
         </is>
@@ -5944,38 +6034,43 @@
       <c r="L2" s="2">
         <v>41</v>
       </c>
-      <c r="M2" s="2">
+      <c r="M2" s="0" t="inlineStr">
+        <is>
+          <t>MEASURED</t>
+        </is>
+      </c>
+      <c r="N2" s="2">
         <v>4</v>
       </c>
-      <c r="N2" s="2">
+      <c r="O2" s="2">
         <v>39508</v>
       </c>
-      <c r="O2" s="3">
+      <c r="P2" s="3">
         <v>790.16</v>
       </c>
-      <c r="P2" s="3">
+      <c r="Q2" s="3">
         <v>3.4286065721184498</v>
       </c>
-      <c r="Q2" s="3">
+      <c r="R2" s="3">
         <v>12.49161094141159</v>
       </c>
-      <c r="R2" s="3">
+      <c r="S2" s="3">
         <v>101.62445254003131</v>
       </c>
-      <c r="S2" s="3">
+      <c r="T2" s="3">
         <v>16.04862513376996</v>
       </c>
-      <c r="T2" s="0" t="inlineStr">
+      <c r="U2" s="0" t="inlineStr">
         <is>
           <t>recursive_skewdct_N1024_20261026/raw_reports/skewdct_50MHz/utilization_hierarchical_post_route.rpt</t>
         </is>
       </c>
-      <c r="U2" s="0" t="inlineStr">
+      <c r="V2" s="0" t="inlineStr">
         <is>
           <t>recursive_skewdct_N1024_20261026/raw_reports/skewdct_50MHz/utilization_hierarchical_post_route.rpt</t>
         </is>
       </c>
-      <c r="V2" s="0" t="inlineStr">
+      <c r="W2" s="0" t="inlineStr">
         <is>
           <t>c64_pipeline_N1024_150MHz_20261026/results/rtl_precision_performance.json</t>
         </is>
@@ -5996,69 +6091,90 @@
       <c r="D3" s="2">
         <v>50</v>
       </c>
-      <c r="E3" s="2">
-        <v>30188</v>
-      </c>
-      <c r="F3" s="2">
-        <v>41987</v>
-      </c>
-      <c r="G3" s="3">
-        <v>9.0</v>
-      </c>
-      <c r="H3" s="2">
-        <v>19</v>
-      </c>
-      <c r="I3" s="2">
-        <v>647</v>
-      </c>
-      <c r="J3" s="2">
-        <v>1098</v>
-      </c>
-      <c r="K3" s="3">
-        <v>2.5</v>
-      </c>
-      <c r="L3" s="2">
-        <v>1</v>
-      </c>
-      <c r="M3" s="2">
+      <c r="E3" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="H3" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="I3" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="J3" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="K3" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L3" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M3" s="0" t="inlineStr">
+        <is>
+          <t>PENDING_REGISTER_IMPLEMENTATION</t>
+        </is>
+      </c>
+      <c r="N3" s="2">
         <v>4</v>
       </c>
-      <c r="N3" s="2">
-        <v>43687</v>
-      </c>
-      <c r="O3" s="3">
-        <v>873.74</v>
+      <c r="O3" s="2">
+        <v>43622</v>
       </c>
       <c r="P3" s="3">
+        <v>872.44</v>
+      </c>
+      <c r="Q3" s="3">
         <v>3.4285470932893625</v>
       </c>
-      <c r="Q3" s="3">
+      <c r="R3" s="3">
         <v>12.490109975036425</v>
       </c>
-      <c r="R3" s="3">
+      <c r="S3" s="3">
         <v>101.60887915401372</v>
       </c>
-      <c r="S3" s="3">
+      <c r="T3" s="3">
         <v>16.04966887517948</v>
       </c>
-      <c r="T3" s="0" t="inlineStr">
-        <is>
-          <t>recursive_skewdct_N1024_20261026/raw_reports/matrixdct_50MHz/utilization_hierarchical_post_route.rpt</t>
-        </is>
-      </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t>recursive_skewdct_N1024_20261026/raw_reports/matrixdct_50MHz/utilization_hierarchical_post_route.rpt</t>
+          <t>matrix_register_20261026/verified_results.json</t>
         </is>
       </c>
       <c r="V3" s="0" t="inlineStr">
         <is>
-          <t>c64_pipeline_N1024_150MHz_20261026/results/rtl_precision_performance.json</t>
+          <t>matrix_register_20261026/verified_results.json</t>
+        </is>
+      </c>
+      <c r="W3" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_20261026/verified_results.json</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V3"/>
+  <autoFilter ref="A1:W3"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Import 50 MHz register-MatrixDCT and standalone-DCT benchmarks
Fill pending MatrixDCT resource and timing fields with supplied results.
Add a standalone-DCT comparison sheet, preserve separate hierarchy scopes,
and retain original CSV/JSON summaries with checksums and evidence notes.

Crosscheck metrics and cycle conversions; correct the derived FF percentage
in analysis while preserving the original summary. No RTL changes.
</commit_message>
<xml_diff>
--- a/docs/benchmarks/MFCC_Benchmark_Summary.xlsx
+++ b/docs/benchmarks/MFCC_Benchmark_Summary.xlsx
@@ -9,12 +9,13 @@
     <sheet name="FFT_Latency" sheetId="5" r:id="rId5"/>
     <sheet name="FFT_Accuracy" sheetId="6" r:id="rId6"/>
     <sheet name="DCT_Comparison" sheetId="7" r:id="rId7"/>
-    <sheet name="Memory_Savings" sheetId="8" r:id="rId8"/>
-    <sheet name="Memory_Regression" sheetId="9" r:id="rId9"/>
-    <sheet name="Timing_Paths" sheetId="10" r:id="rId10"/>
-    <sheet name="Coverage" sheetId="11" r:id="rId11"/>
-    <sheet name="Sources" sheetId="12" r:id="rId12"/>
-    <sheet name="Readme" sheetId="13" r:id="rId13"/>
+    <sheet name="DCT_Standalone" sheetId="8" r:id="rId8"/>
+    <sheet name="Memory_Savings" sheetId="9" r:id="rId9"/>
+    <sheet name="Memory_Regression" sheetId="10" r:id="rId10"/>
+    <sheet name="Timing_Paths" sheetId="11" r:id="rId11"/>
+    <sheet name="Coverage" sheetId="12" r:id="rId12"/>
+    <sheet name="Sources" sheetId="13" r:id="rId13"/>
+    <sheet name="Readme" sheetId="14" r:id="rId14"/>
   </sheets>
 </workbook>
 </file>
@@ -86,7 +87,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P25"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -673,49 +674,33 @@
       <c r="E10" s="2">
         <v>64</v>
       </c>
-      <c r="F10" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G10" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H10" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I10" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J10" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K10" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L10" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M10" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F10" s="2">
+        <v>1749</v>
+      </c>
+      <c r="G10" s="3">
+        <v>1.49</v>
+      </c>
+      <c r="H10" s="2">
+        <v>2584</v>
+      </c>
+      <c r="I10" s="3">
+        <v>1.1</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="L10" s="2">
+        <v>1</v>
+      </c>
+      <c r="M10" s="3">
+        <v>0.08</v>
       </c>
       <c r="N10" s="0" t="inlineStr">
         <is>
-          <t>Register/LUT RTL; hardware reimplementation pending</t>
+          <t>OOC post-route; user-supplied summary; raw report not supplied</t>
         </is>
       </c>
       <c r="O10" s="3">
@@ -723,7 +708,7 @@
       </c>
       <c r="P10" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/verified_results.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
     </row>
@@ -921,49 +906,33 @@
       <c r="E14" s="2">
         <v>64</v>
       </c>
-      <c r="F14" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G14" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H14" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I14" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J14" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K14" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L14" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M14" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="F14" s="2">
+        <v>30110</v>
+      </c>
+      <c r="G14" s="3">
+        <v>25.71</v>
+      </c>
+      <c r="H14" s="2">
+        <v>43473</v>
+      </c>
+      <c r="I14" s="3">
+        <v>18.56</v>
+      </c>
+      <c r="J14" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="K14" s="3">
+        <v>4.51</v>
+      </c>
+      <c r="L14" s="2">
+        <v>19</v>
+      </c>
+      <c r="M14" s="3">
+        <v>1.52</v>
       </c>
       <c r="N14" s="0" t="inlineStr">
         <is>
-          <t>Register/LUT RTL; hardware reimplementation pending</t>
+          <t>OOC post-route; user-supplied summary; raw report not supplied</t>
         </is>
       </c>
       <c r="O14" s="3">
@@ -971,7 +940,7 @@
       </c>
       <c r="P14" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/verified_results.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
     </row>
@@ -1517,13 +1486,647 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="0" t="inlineStr">
+        <is>
+          <t>MatrixDCT</t>
+        </is>
+      </c>
+      <c r="B24" s="0" t="inlineStr">
+        <is>
+          <t>Standalone DCT</t>
+        </is>
+      </c>
+      <c r="C24" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D24" s="2">
+        <v>50</v>
+      </c>
+      <c r="E24" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F24" s="2">
+        <v>1847</v>
+      </c>
+      <c r="G24" s="3">
+        <v>1.58</v>
+      </c>
+      <c r="H24" s="2">
+        <v>2717</v>
+      </c>
+      <c r="I24" s="3">
+        <v>1.16</v>
+      </c>
+      <c r="J24" s="2">
+        <v>0</v>
+      </c>
+      <c r="K24" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="L24" s="2">
+        <v>1</v>
+      </c>
+      <c r="M24" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="N24" s="0" t="inlineStr">
+        <is>
+          <t>OOC post-route; user-supplied summary; raw report not supplied</t>
+        </is>
+      </c>
+      <c r="O24" s="2">
+        <v>20</v>
+      </c>
+      <c r="P24" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_50MHz_20261027/results.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0" t="inlineStr">
+        <is>
+          <t>SkewDCT</t>
+        </is>
+      </c>
+      <c r="B25" s="0" t="inlineStr">
+        <is>
+          <t>Standalone DCT</t>
+        </is>
+      </c>
+      <c r="C25" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="D25" s="2">
+        <v>50</v>
+      </c>
+      <c r="E25" s="0" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F25" s="2">
+        <v>5113</v>
+      </c>
+      <c r="G25" s="3">
+        <v>4.37</v>
+      </c>
+      <c r="H25" s="2">
+        <v>12378</v>
+      </c>
+      <c r="I25" s="3">
+        <v>5.28</v>
+      </c>
+      <c r="J25" s="2">
+        <v>0</v>
+      </c>
+      <c r="K25" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="L25" s="2">
+        <v>41</v>
+      </c>
+      <c r="M25" s="3">
+        <v>3.29</v>
+      </c>
+      <c r="N25" s="0" t="inlineStr">
+        <is>
+          <t>OOC post-route; user-supplied summary; raw report not supplied</t>
+        </is>
+      </c>
+      <c r="O25" s="2">
+        <v>20</v>
+      </c>
+      <c r="P25" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_50MHz_20261027/results.json</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P23"/>
+  <autoFilter ref="A1:P25"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:K12"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="26" customWidth="1"/>
+    <col min="8" max="8" width="25" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="28" customWidth="1"/>
+    <col min="11" max="11" width="65" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FFT N</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Output lanes</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Stalls</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Frames</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Before cycles</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>After cycles</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Before batch us at 50MHz</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>After batch us at 50MHz</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Cycle change %</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Mismatches to own reference</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2">
+        <v>16</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1</v>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D2" s="2">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2">
+        <v>1226</v>
+      </c>
+      <c r="F2" s="2">
+        <v>1226</v>
+      </c>
+      <c r="G2" s="3">
+        <v>24.52</v>
+      </c>
+      <c r="H2" s="3">
+        <v>24.52</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0</v>
+      </c>
+      <c r="K2" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2">
+        <v>32</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D3" s="2">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1393</v>
+      </c>
+      <c r="F3" s="2">
+        <v>1407</v>
+      </c>
+      <c r="G3" s="3">
+        <v>27.86</v>
+      </c>
+      <c r="H3" s="3">
+        <v>28.14</v>
+      </c>
+      <c r="I3" s="3">
+        <v>1.0050251256281406</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0</v>
+      </c>
+      <c r="K3" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2">
+        <v>64</v>
+      </c>
+      <c r="B4" s="2">
+        <v>1</v>
+      </c>
+      <c r="C4" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D4" s="2">
+        <v>4</v>
+      </c>
+      <c r="E4" s="2">
+        <v>2757</v>
+      </c>
+      <c r="F4" s="2">
+        <v>2537</v>
+      </c>
+      <c r="G4" s="3">
+        <v>55.14</v>
+      </c>
+      <c r="H4" s="3">
+        <v>50.74</v>
+      </c>
+      <c r="I4" s="3">
+        <v>-7.979688066739208</v>
+      </c>
+      <c r="J4" s="2">
+        <v>0</v>
+      </c>
+      <c r="K4" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>128</v>
+      </c>
+      <c r="B5" s="2">
+        <v>1</v>
+      </c>
+      <c r="C5" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D5" s="2">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2">
+        <v>4304</v>
+      </c>
+      <c r="F5" s="2">
+        <v>4304</v>
+      </c>
+      <c r="G5" s="3">
+        <v>86.08</v>
+      </c>
+      <c r="H5" s="3">
+        <v>86.08</v>
+      </c>
+      <c r="I5" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0</v>
+      </c>
+      <c r="K5" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>256</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1</v>
+      </c>
+      <c r="C6" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D6" s="2">
+        <v>4</v>
+      </c>
+      <c r="E6" s="2">
+        <v>6853</v>
+      </c>
+      <c r="F6" s="2">
+        <v>6838</v>
+      </c>
+      <c r="G6" s="3">
+        <v>137.06</v>
+      </c>
+      <c r="H6" s="3">
+        <v>136.76</v>
+      </c>
+      <c r="I6" s="3">
+        <v>-0.2188822413541515</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0</v>
+      </c>
+      <c r="K6" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>512</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
+      <c r="C7" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D7" s="2">
+        <v>4</v>
+      </c>
+      <c r="E7" s="2">
+        <v>12990</v>
+      </c>
+      <c r="F7" s="2">
+        <v>13950</v>
+      </c>
+      <c r="G7" s="3">
+        <v>259.8</v>
+      </c>
+      <c r="H7" s="3">
+        <v>279.0</v>
+      </c>
+      <c r="I7" s="3">
+        <v>7.390300230946882</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0</v>
+      </c>
+      <c r="K7" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>1024</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D8" s="2">
+        <v>4</v>
+      </c>
+      <c r="E8" s="2">
+        <v>41365</v>
+      </c>
+      <c r="F8" s="2">
+        <v>37307</v>
+      </c>
+      <c r="G8" s="3">
+        <v>827.3</v>
+      </c>
+      <c r="H8" s="3">
+        <v>746.14</v>
+      </c>
+      <c r="I8" s="3">
+        <v>-9.810226036504291</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0</v>
+      </c>
+      <c r="K8" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>2048</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1</v>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D9" s="2">
+        <v>4</v>
+      </c>
+      <c r="E9" s="2">
+        <v>65677</v>
+      </c>
+      <c r="F9" s="2">
+        <v>65677</v>
+      </c>
+      <c r="G9" s="3">
+        <v>1313.54</v>
+      </c>
+      <c r="H9" s="3">
+        <v>1313.54</v>
+      </c>
+      <c r="I9" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0</v>
+      </c>
+      <c r="K9" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>128</v>
+      </c>
+      <c r="B10" s="2">
+        <v>64</v>
+      </c>
+      <c r="C10" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D10" s="2">
+        <v>4</v>
+      </c>
+      <c r="E10" s="2">
+        <v>4233</v>
+      </c>
+      <c r="F10" s="2">
+        <v>4233</v>
+      </c>
+      <c r="G10" s="3">
+        <v>84.66</v>
+      </c>
+      <c r="H10" s="3">
+        <v>84.66</v>
+      </c>
+      <c r="I10" s="3">
+        <v>0.0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>512</v>
+      </c>
+      <c r="B11" s="2">
+        <v>64</v>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="D11" s="2">
+        <v>16</v>
+      </c>
+      <c r="E11" s="2">
+        <v>47658</v>
+      </c>
+      <c r="F11" s="2">
+        <v>51711</v>
+      </c>
+      <c r="G11" s="3">
+        <v>953.16</v>
+      </c>
+      <c r="H11" s="3">
+        <v>1034.22</v>
+      </c>
+      <c r="I11" s="3">
+        <v>8.504343447060304</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0</v>
+      </c>
+      <c r="K11" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
+        <v>512</v>
+      </c>
+      <c r="B12" s="2">
+        <v>64</v>
+      </c>
+      <c r="C12" s="0" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="D12" s="2">
+        <v>16</v>
+      </c>
+      <c r="E12" s="2">
+        <v>47210</v>
+      </c>
+      <c r="F12" s="2">
+        <v>51258</v>
+      </c>
+      <c r="G12" s="3">
+        <v>944.2</v>
+      </c>
+      <c r="H12" s="3">
+        <v>1025.16</v>
+      </c>
+      <c r="I12" s="3">
+        <v>8.574454564710866</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0</v>
+      </c>
+      <c r="K12" s="0" t="inlineStr">
+        <is>
+          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K12"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:K21"/>
   <sheetFormatPr defaultRowHeight="30"/>
@@ -2464,9 +3067,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2681,36 +3284,58 @@
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>Six unit cases; twenty MFCC configurations</t>
+          <t>Six unit cases; twenty MFCC configurations; supplied 50 MHz OOC result</t>
         </is>
       </c>
       <c r="C10" s="0" t="inlineStr">
         <is>
-          <t>Simulation passes; new physical resource/timing mapping pending</t>
+          <t>Local regression passes; latest hardware fields supplied in result summaries</t>
         </is>
       </c>
       <c r="D10" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/README.md</t>
+          <t>matrix_register_50MHz_20261027/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="0" t="inlineStr">
+        <is>
+          <t>Standalone DCT comparison</t>
+        </is>
+      </c>
+      <c r="B11" s="0" t="inlineStr">
+        <is>
+          <t>64-point register MatrixDCT versus recursive SkewDCT; 50 MHz</t>
+        </is>
+      </c>
+      <c r="C11" s="0" t="inlineStr">
+        <is>
+          <t>Included; resources, first/final latency and WNS/WHS; supplied summaries</t>
+        </is>
+      </c>
+      <c r="D11" s="0" t="inlineStr">
+        <is>
+          <t>dct/DCT_Standalone.csv</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D10"/>
+  <autoFilter ref="A1:D11"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="3" max="3" width="28" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
     <col min="6" max="6" width="15" customWidth="1"/>
     <col min="7" max="7" width="65" customWidth="1"/>
   </cols>
@@ -2728,7 +3353,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Archive filename</t>
+          <t>Archive or summary filename</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -2738,7 +3363,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Archive SHA256</t>
+          <t>SHA256</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -2962,15 +3587,85 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_20261027_json</t>
+        </is>
+      </c>
+      <c r="B8" s="0" t="inlineStr">
+        <is>
+          <t>Register MatrixDCT and recursive SkewDCT, 50 MHz</t>
+        </is>
+      </c>
+      <c r="C8" s="0" t="inlineStr">
+        <is>
+          <t>results.json</t>
+        </is>
+      </c>
+      <c r="D8" s="2">
+        <v>2413</v>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
+        <is>
+          <t>193620521ac3fd20b196d5be97bd3ed02b220c8446d9844450d296192b4ed93c</t>
+        </is>
+      </c>
+      <c r="F8" s="0" t="inlineStr">
+        <is>
+          <t>0dce6b054028ff37c3158adc0184acc030211d0e</t>
+        </is>
+      </c>
+      <c r="G8" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_50MHz_20261027</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_20261027_csv</t>
+        </is>
+      </c>
+      <c r="B9" s="0" t="inlineStr">
+        <is>
+          <t>Register MatrixDCT and recursive SkewDCT, 50 MHz</t>
+        </is>
+      </c>
+      <c r="C9" s="0" t="inlineStr">
+        <is>
+          <t>results.csv</t>
+        </is>
+      </c>
+      <c r="D9" s="2">
+        <v>766</v>
+      </c>
+      <c r="E9" s="0" t="inlineStr">
+        <is>
+          <t>a98e913348e6c9c73f8827a10f9ad22a301423735e3c70e82f2e09a71315b348</t>
+        </is>
+      </c>
+      <c r="F9" s="0" t="inlineStr">
+        <is>
+          <t>0dce6b054028ff37c3158adc0184acc030211d0e</t>
+        </is>
+      </c>
+      <c r="G9" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_50MHz_20261027</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:G7"/>
+  <autoFilter ref="A1:G9"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr defaultRowHeight="30"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -2997,156 +3692,180 @@
       </c>
       <c r="B2" s="0" t="inlineStr">
         <is>
-          <t>Current MatrixDCT uses register/LUT storage. Its new resource and timing fields are pending, not copied from the obsolete BRAM implementation. Latest verified N1024 batch: 43622 cycles. Original hardware reports remain historical evidence.</t>
+          <t>Register/LUT MatrixDCT hardware fields now use supplied 2026-10-27 50 MHz OOC post-route summaries. Original BRAM measurements remain historical. New whole-MFCC resources: 30110 LUT, 43473 FF, 6.5 BRAM, 19 DSP; batch 43622 cycles.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="0" t="inlineStr">
         <is>
-          <t>Selection rule</t>
+          <t>Standalone DCT scope</t>
         </is>
       </c>
       <c r="B3" s="0" t="inlineStr">
         <is>
-          <t>Keep the latest valid value per test project and configuration. Architecture/pipeline/version names are not separate test projects.</t>
+          <t>Standalone top-level resources and latency are separate from the inclusive MFCC DCT hierarchy. Both standalone DCTs report zero BRAM; MatrixDCT uses one DSP and SkewDCT 41, so arithmetic parallelism remains different.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="0" t="inlineStr">
         <is>
-          <t>Configuration key</t>
+          <t>Supplied result evidence</t>
         </is>
       </c>
       <c r="B4" s="0" t="inlineStr">
         <is>
-          <t>Project, backend under comparison, N, frequency, output lanes, frame count and stall condition identify a case. Inclusive hierarchy scope is retained.</t>
+          <t>CSV and JSON summaries agree; original Vivado reports and coefficient dumps were not supplied. Positive WNS/WHS are user-reported; TNS and setup/hold failure counts remain blank. No new whole-MFCC SkewDCT implementation results were supplied.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="0" t="inlineStr">
         <is>
-          <t>Partial updates</t>
+          <t>Selection rule</t>
         </is>
       </c>
       <c r="B5" s="0" t="inlineStr">
         <is>
-          <t>Refresh metrics separately: a 150 MHz resource update does not invent new 50/100 MHz resources. Unchanged metrics use the latest available reports. Runtime cycle counts use the latest matching regression and are converted by frequency.</t>
+          <t>Keep the latest valid value per test project and configuration. Architecture/pipeline/version names are not separate test projects.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="0" t="inlineStr">
         <is>
-          <t>Sources</t>
+          <t>Configuration key</t>
         </is>
       </c>
       <c r="B6" s="0" t="inlineStr">
         <is>
-          <t>Source paths in tables and JSON are relative to docs/benchmarks/. Per-metric source columns identify the original evidence; different metric groups can come from different packages.</t>
+          <t>Project, backend under comparison, N, frequency, output lanes, frame count and stall condition identify a case. Inclusive hierarchy scope is retained.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="0" t="inlineStr">
         <is>
-          <t>Resource priority</t>
+          <t>Partial updates</t>
         </is>
       </c>
       <c r="B7" s="0" t="inlineStr">
         <is>
-          <t>LUT, FF, BRAM and DSP appear first. DCT/C64/SkewDCT8 hierarchy rows are already included in parent totals.</t>
+          <t>Refresh metrics separately: a 150 MHz resource update does not invent new 50/100 MHz resources. Unchanged metrics use the latest available reports. Runtime cycle counts use the latest matching regression and are converted by frequency.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="0" t="inlineStr">
         <is>
-          <t>BRAM unit</t>
+          <t>Sources</t>
         </is>
       </c>
       <c r="B8" s="0" t="inlineStr">
         <is>
-          <t>One BRAM tile is a 36 Kb equivalent; each RAMB18 counts as 0.5 tile.</t>
+          <t>Source paths in tables and JSON are relative to docs/benchmarks/. Per-metric source columns identify the original evidence; different metric groups can come from different packages.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="0" t="inlineStr">
         <is>
-          <t>FFT evidence</t>
+          <t>Resource priority</t>
         </is>
       </c>
       <c r="B9" s="0" t="inlineStr">
         <is>
-          <t>XFFT resource reports use fixed-size cores and a 10 ns synthesis clock; custom FFT resources use a shared runtime core after routing at 20 ns. The 64..2048 XFFT latency numbers use runtime_2048. These attributes remain source metadata, not version-specific result rows.</t>
+          <t>LUT, FF, BRAM and DSP appear first. DCT/C64/SkewDCT8 hierarchy rows are already included in parent totals.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="0" t="inlineStr">
         <is>
-          <t>FFT 16-point counting</t>
+          <t>BRAM unit</t>
         </is>
       </c>
       <c r="B10" s="0" t="inlineStr">
         <is>
-          <t>Latest reported custom complete-frame latency is 82 cycles; its accompanying regression records 83. The primary table retains the latest reported value and marks this counting discrepancy.</t>
+          <t>One BRAM tile is a 36 Kb equivalent; each RAMB18 counts as 0.5 tile.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="0" t="inlineStr">
         <is>
-          <t>FFT first output</t>
+          <t>FFT evidence</t>
         </is>
       </c>
       <c r="B11" s="0" t="inlineStr">
         <is>
-          <t>First-output cycles are taken from the latest package reporting that metric (2026-10-22); complete-frame comparisons are updated by the 2026-10-25 package.</t>
+          <t>XFFT resource reports use fixed-size cores and a 10 ns synthesis clock; custom FFT resources use a shared runtime core after routing at 20 ns. The 64..2048 XFFT latency numbers use runtime_2048. These attributes remain source metadata, not version-specific result rows.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="0" t="inlineStr">
         <is>
-          <t>Timing/accuracy scope</t>
+          <t>FFT 16-point counting</t>
         </is>
       </c>
       <c r="B12" s="0" t="inlineStr">
         <is>
-          <t>Times are RTL cycles divided by MHz, not board/PS/DMA measurements. Four-frame averages are not independently measured single-frame latency or steady-state II. MFCC reference errors do not isolate DCT error or recognition accuracy.</t>
+          <t>Latest reported custom complete-frame latency is 82 cycles; its accompanying regression records 83. The primary table retains the latest reported value and marks this counting discrepancy.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="0" t="inlineStr">
         <is>
-          <t>History</t>
+          <t>FFT first output</t>
         </is>
       </c>
       <c r="B13" s="0" t="inlineStr">
         <is>
-          <t>Superseded values remain in immutable original reports for traceability, outside primary tables. The explicit paired memory before/after experiment retains both required comparison sides.</t>
+          <t>First-output cycles are taken from the latest package reporting that metric (2026-10-22); complete-frame comparisons are updated by the 2026-10-25 package.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="0" t="inlineStr">
         <is>
+          <t>Timing/accuracy scope</t>
+        </is>
+      </c>
+      <c r="B14" s="0" t="inlineStr">
+        <is>
+          <t>Times are RTL cycles divided by MHz, not board/PS/DMA measurements. Four-frame averages are not independently measured single-frame latency or steady-state II. MFCC reference errors do not isolate DCT error or recognition accuracy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="0" t="inlineStr">
+        <is>
+          <t>History</t>
+        </is>
+      </c>
+      <c r="B15" s="0" t="inlineStr">
+        <is>
+          <t>Superseded values remain in immutable original reports for traceability, outside primary tables. The explicit paired memory before/after experiment retains both required comparison sides.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="0" t="inlineStr">
+        <is>
           <t>200 MHz status</t>
         </is>
       </c>
-      <c r="B14" s="0" t="inlineStr">
+      <c r="B16" s="0" t="inlineStr">
         <is>
           <t>Not measured for the latest RTL. Frozen-route estimate is approximately -1.409 ns. The old 200 MHz run was interrupted during placement and is not a pass/fail result.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B14"/>
+  <autoFilter ref="A1:B16"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
 </file>
@@ -3366,7 +4085,7 @@
       </c>
       <c r="V2" s="0" t="inlineStr">
         <is>
-          <t>c64_pipeline_N1024_150MHz_20261026/results/rtl_precision_performance.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
     </row>
@@ -3444,7 +4163,7 @@
       </c>
       <c r="V3" s="0" t="inlineStr">
         <is>
-          <t>c64_pipeline_N1024_150MHz_20261026/results/rtl_precision_performance.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
     </row>
@@ -3522,7 +4241,7 @@
       </c>
       <c r="V4" s="0" t="inlineStr">
         <is>
-          <t>c64_pipeline_N1024_150MHz_20261026/results/rtl_precision_performance.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
     </row>
@@ -3547,54 +4266,42 @@
       <c r="F5" s="2">
         <v>50</v>
       </c>
-      <c r="G5" s="0" t="inlineStr">
+      <c r="G5" s="2">
+        <v>30110</v>
+      </c>
+      <c r="H5" s="2">
+        <v>43473</v>
+      </c>
+      <c r="I5" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="J5" s="2">
+        <v>19</v>
+      </c>
+      <c r="K5" s="3">
+        <v>8.235</v>
+      </c>
+      <c r="L5" s="0" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="H5" s="0" t="inlineStr">
+      <c r="M5" s="0" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="I5" s="0" t="inlineStr">
+      <c r="N5" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="O5" s="0" t="inlineStr">
         <is>
           <t/>
         </is>
       </c>
-      <c r="J5" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K5" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L5" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M5" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N5" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O5" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
       <c r="P5" s="0" t="inlineStr">
         <is>
-          <t>PENDING_REGISTER_IMPLEMENTATION</t>
+          <t>PASS_REPORTED_WNS_WHS</t>
         </is>
       </c>
       <c r="Q5" s="2">
@@ -3608,17 +4315,17 @@
       </c>
       <c r="T5" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/verified_results.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
       <c r="U5" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/verified_results.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
       <c r="V5" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/verified_results.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
     </row>
@@ -6036,7 +6743,7 @@
       </c>
       <c r="M2" s="0" t="inlineStr">
         <is>
-          <t>MEASURED</t>
+          <t>MEASURED_PREVIOUS_REPORT</t>
         </is>
       </c>
       <c r="N2" s="2">
@@ -6052,10 +6759,10 @@
         <v>3.4286065721184498</v>
       </c>
       <c r="R2" s="3">
-        <v>12.49161094141159</v>
+        <v>12.491610941411583</v>
       </c>
       <c r="S2" s="3">
-        <v>101.62445254003131</v>
+        <v>101.62445254003143</v>
       </c>
       <c r="T2" s="3">
         <v>16.04862513376996</v>
@@ -6072,7 +6779,7 @@
       </c>
       <c r="W2" s="0" t="inlineStr">
         <is>
-          <t>c64_pipeline_N1024_150MHz_20261026/results/rtl_precision_performance.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
     </row>
@@ -6091,49 +6798,33 @@
       <c r="D3" s="2">
         <v>50</v>
       </c>
-      <c r="E3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="F3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="G3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="H3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="I3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="J3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="K3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="L3" s="0" t="inlineStr">
-        <is>
-          <t/>
-        </is>
+      <c r="E3" s="2">
+        <v>30110</v>
+      </c>
+      <c r="F3" s="2">
+        <v>43473</v>
+      </c>
+      <c r="G3" s="3">
+        <v>6.5</v>
+      </c>
+      <c r="H3" s="2">
+        <v>19</v>
+      </c>
+      <c r="I3" s="2">
+        <v>1749</v>
+      </c>
+      <c r="J3" s="2">
+        <v>2584</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0</v>
+      </c>
+      <c r="L3" s="2">
+        <v>1</v>
       </c>
       <c r="M3" s="0" t="inlineStr">
         <is>
-          <t>PENDING_REGISTER_IMPLEMENTATION</t>
+          <t>REPORTED_POST_ROUTE</t>
         </is>
       </c>
       <c r="N3" s="2">
@@ -6146,30 +6837,30 @@
         <v>872.44</v>
       </c>
       <c r="Q3" s="3">
-        <v>3.4285470932893625</v>
+        <v>3.428547093289361</v>
       </c>
       <c r="R3" s="3">
-        <v>12.490109975036425</v>
+        <v>12.490109975036418</v>
       </c>
       <c r="S3" s="3">
-        <v>101.60887915401372</v>
+        <v>101.60887915401383</v>
       </c>
       <c r="T3" s="3">
-        <v>16.04966887517948</v>
+        <v>16.049668875179485</v>
       </c>
       <c r="U3" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/verified_results.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
       <c r="V3" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/verified_results.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
       <c r="W3" s="0" t="inlineStr">
         <is>
-          <t>matrix_register_20261026/verified_results.json</t>
+          <t>matrix_register_50MHz_20261027/results.json</t>
         </is>
       </c>
     </row>
@@ -6180,6 +6871,233 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:P3"/>
+  <sheetFormatPr defaultRowHeight="30"/>
+  <cols>
+    <col min="1" max="1" width="15" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="15" customWidth="1"/>
+    <col min="8" max="8" width="15" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="15" customWidth="1"/>
+    <col min="11" max="11" width="21" customWidth="1"/>
+    <col min="12" max="12" width="21" customWidth="1"/>
+    <col min="13" max="13" width="17" customWidth="1"/>
+    <col min="14" max="14" width="17" customWidth="1"/>
+    <col min="15" max="15" width="15" customWidth="1"/>
+    <col min="16" max="16" width="65" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Backend</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>DCT points</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>MHz</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>LUT</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>FF</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>BRAM tiles</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>WNS ns</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>WHS ns</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>First output cycles</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Final output cycles</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>First output us</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Final output us</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Tested commit</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t>MatrixDCT</t>
+        </is>
+      </c>
+      <c r="B2" s="2">
+        <v>64</v>
+      </c>
+      <c r="C2" s="2">
+        <v>50</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1847</v>
+      </c>
+      <c r="E2" s="2">
+        <v>2717</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <v>1</v>
+      </c>
+      <c r="H2" s="3">
+        <v>12.74</v>
+      </c>
+      <c r="I2" s="3">
+        <v>0.067</v>
+      </c>
+      <c r="J2" s="0" t="inlineStr">
+        <is>
+          <t>PASS_REPORTED_WNS_WHS</t>
+        </is>
+      </c>
+      <c r="K2" s="2">
+        <v>4289</v>
+      </c>
+      <c r="L2" s="2">
+        <v>4352</v>
+      </c>
+      <c r="M2" s="3">
+        <v>85.78</v>
+      </c>
+      <c r="N2" s="3">
+        <v>87.04</v>
+      </c>
+      <c r="O2" s="0" t="inlineStr">
+        <is>
+          <t>0dce6b054028ff37c3158adc0184acc030211d0e</t>
+        </is>
+      </c>
+      <c r="P2" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_50MHz_20261027/results.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="0" t="inlineStr">
+        <is>
+          <t>SkewDCT</t>
+        </is>
+      </c>
+      <c r="B3" s="2">
+        <v>64</v>
+      </c>
+      <c r="C3" s="2">
+        <v>50</v>
+      </c>
+      <c r="D3" s="2">
+        <v>5113</v>
+      </c>
+      <c r="E3" s="2">
+        <v>12378</v>
+      </c>
+      <c r="F3" s="2">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>41</v>
+      </c>
+      <c r="H3" s="3">
+        <v>14.342</v>
+      </c>
+      <c r="I3" s="3">
+        <v>0.011</v>
+      </c>
+      <c r="J3" s="0" t="inlineStr">
+        <is>
+          <t>PASS_REPORTED_WNS_WHS</t>
+        </is>
+      </c>
+      <c r="K3" s="2">
+        <v>175</v>
+      </c>
+      <c r="L3" s="2">
+        <v>238</v>
+      </c>
+      <c r="M3" s="3">
+        <v>3.5</v>
+      </c>
+      <c r="N3" s="3">
+        <v>4.76</v>
+      </c>
+      <c r="O3" s="0" t="inlineStr">
+        <is>
+          <t>0dce6b054028ff37c3158adc0184acc030211d0e</t>
+        </is>
+      </c>
+      <c r="P3" s="0" t="inlineStr">
+        <is>
+          <t>matrix_register_50MHz_20261027/results.json</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P3"/>
+  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="30"/>
@@ -6348,514 +7266,4 @@
   <autoFilter ref="A1:F6"/>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:K12"/>
-  <sheetFormatPr defaultRowHeight="30"/>
-  <cols>
-    <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="26" customWidth="1"/>
-    <col min="8" max="8" width="25" customWidth="1"/>
-    <col min="9" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="28" customWidth="1"/>
-    <col min="11" max="11" width="65" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>FFT N</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Output lanes</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Stalls</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Frames</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Before cycles</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>After cycles</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Before batch us at 50MHz</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>After batch us at 50MHz</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Cycle change %</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Mismatches to own reference</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Source</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2">
-        <v>16</v>
-      </c>
-      <c r="B2" s="2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D2" s="2">
-        <v>4</v>
-      </c>
-      <c r="E2" s="2">
-        <v>1226</v>
-      </c>
-      <c r="F2" s="2">
-        <v>1226</v>
-      </c>
-      <c r="G2" s="3">
-        <v>24.52</v>
-      </c>
-      <c r="H2" s="3">
-        <v>24.52</v>
-      </c>
-      <c r="I2" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="J2" s="2">
-        <v>0</v>
-      </c>
-      <c r="K2" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2">
-        <v>32</v>
-      </c>
-      <c r="B3" s="2">
-        <v>1</v>
-      </c>
-      <c r="C3" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D3" s="2">
-        <v>4</v>
-      </c>
-      <c r="E3" s="2">
-        <v>1393</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1407</v>
-      </c>
-      <c r="G3" s="3">
-        <v>27.86</v>
-      </c>
-      <c r="H3" s="3">
-        <v>28.14</v>
-      </c>
-      <c r="I3" s="3">
-        <v>1.0050251256281406</v>
-      </c>
-      <c r="J3" s="2">
-        <v>0</v>
-      </c>
-      <c r="K3" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2">
-        <v>64</v>
-      </c>
-      <c r="B4" s="2">
-        <v>1</v>
-      </c>
-      <c r="C4" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D4" s="2">
-        <v>4</v>
-      </c>
-      <c r="E4" s="2">
-        <v>2757</v>
-      </c>
-      <c r="F4" s="2">
-        <v>2537</v>
-      </c>
-      <c r="G4" s="3">
-        <v>55.14</v>
-      </c>
-      <c r="H4" s="3">
-        <v>50.74</v>
-      </c>
-      <c r="I4" s="3">
-        <v>-7.979688066739208</v>
-      </c>
-      <c r="J4" s="2">
-        <v>0</v>
-      </c>
-      <c r="K4" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2">
-        <v>128</v>
-      </c>
-      <c r="B5" s="2">
-        <v>1</v>
-      </c>
-      <c r="C5" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D5" s="2">
-        <v>4</v>
-      </c>
-      <c r="E5" s="2">
-        <v>4304</v>
-      </c>
-      <c r="F5" s="2">
-        <v>4304</v>
-      </c>
-      <c r="G5" s="3">
-        <v>86.08</v>
-      </c>
-      <c r="H5" s="3">
-        <v>86.08</v>
-      </c>
-      <c r="I5" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="J5" s="2">
-        <v>0</v>
-      </c>
-      <c r="K5" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2">
-        <v>256</v>
-      </c>
-      <c r="B6" s="2">
-        <v>1</v>
-      </c>
-      <c r="C6" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D6" s="2">
-        <v>4</v>
-      </c>
-      <c r="E6" s="2">
-        <v>6853</v>
-      </c>
-      <c r="F6" s="2">
-        <v>6838</v>
-      </c>
-      <c r="G6" s="3">
-        <v>137.06</v>
-      </c>
-      <c r="H6" s="3">
-        <v>136.76</v>
-      </c>
-      <c r="I6" s="3">
-        <v>-0.2188822413541515</v>
-      </c>
-      <c r="J6" s="2">
-        <v>0</v>
-      </c>
-      <c r="K6" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2">
-        <v>512</v>
-      </c>
-      <c r="B7" s="2">
-        <v>1</v>
-      </c>
-      <c r="C7" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D7" s="2">
-        <v>4</v>
-      </c>
-      <c r="E7" s="2">
-        <v>12990</v>
-      </c>
-      <c r="F7" s="2">
-        <v>13950</v>
-      </c>
-      <c r="G7" s="3">
-        <v>259.8</v>
-      </c>
-      <c r="H7" s="3">
-        <v>279.0</v>
-      </c>
-      <c r="I7" s="3">
-        <v>7.390300230946882</v>
-      </c>
-      <c r="J7" s="2">
-        <v>0</v>
-      </c>
-      <c r="K7" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2">
-        <v>1024</v>
-      </c>
-      <c r="B8" s="2">
-        <v>1</v>
-      </c>
-      <c r="C8" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D8" s="2">
-        <v>4</v>
-      </c>
-      <c r="E8" s="2">
-        <v>41365</v>
-      </c>
-      <c r="F8" s="2">
-        <v>37307</v>
-      </c>
-      <c r="G8" s="3">
-        <v>827.3</v>
-      </c>
-      <c r="H8" s="3">
-        <v>746.14</v>
-      </c>
-      <c r="I8" s="3">
-        <v>-9.810226036504291</v>
-      </c>
-      <c r="J8" s="2">
-        <v>0</v>
-      </c>
-      <c r="K8" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2">
-        <v>2048</v>
-      </c>
-      <c r="B9" s="2">
-        <v>1</v>
-      </c>
-      <c r="C9" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D9" s="2">
-        <v>4</v>
-      </c>
-      <c r="E9" s="2">
-        <v>65677</v>
-      </c>
-      <c r="F9" s="2">
-        <v>65677</v>
-      </c>
-      <c r="G9" s="3">
-        <v>1313.54</v>
-      </c>
-      <c r="H9" s="3">
-        <v>1313.54</v>
-      </c>
-      <c r="I9" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="J9" s="2">
-        <v>0</v>
-      </c>
-      <c r="K9" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2">
-        <v>128</v>
-      </c>
-      <c r="B10" s="2">
-        <v>64</v>
-      </c>
-      <c r="C10" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D10" s="2">
-        <v>4</v>
-      </c>
-      <c r="E10" s="2">
-        <v>4233</v>
-      </c>
-      <c r="F10" s="2">
-        <v>4233</v>
-      </c>
-      <c r="G10" s="3">
-        <v>84.66</v>
-      </c>
-      <c r="H10" s="3">
-        <v>84.66</v>
-      </c>
-      <c r="I10" s="3">
-        <v>0.0</v>
-      </c>
-      <c r="J10" s="2">
-        <v>0</v>
-      </c>
-      <c r="K10" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2">
-        <v>512</v>
-      </c>
-      <c r="B11" s="2">
-        <v>64</v>
-      </c>
-      <c r="C11" s="0" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="D11" s="2">
-        <v>16</v>
-      </c>
-      <c r="E11" s="2">
-        <v>47658</v>
-      </c>
-      <c r="F11" s="2">
-        <v>51711</v>
-      </c>
-      <c r="G11" s="3">
-        <v>953.16</v>
-      </c>
-      <c r="H11" s="3">
-        <v>1034.22</v>
-      </c>
-      <c r="I11" s="3">
-        <v>8.504343447060304</v>
-      </c>
-      <c r="J11" s="2">
-        <v>0</v>
-      </c>
-      <c r="K11" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2">
-        <v>512</v>
-      </c>
-      <c r="B12" s="2">
-        <v>64</v>
-      </c>
-      <c r="C12" s="0" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="D12" s="2">
-        <v>16</v>
-      </c>
-      <c r="E12" s="2">
-        <v>47210</v>
-      </c>
-      <c r="F12" s="2">
-        <v>51258</v>
-      </c>
-      <c r="G12" s="3">
-        <v>944.2</v>
-      </c>
-      <c r="H12" s="3">
-        <v>1025.16</v>
-      </c>
-      <c r="I12" s="3">
-        <v>8.574454564710866</v>
-      </c>
-      <c r="J12" s="2">
-        <v>0</v>
-      </c>
-      <c r="K12" s="0" t="inlineStr">
-        <is>
-          <t>evidence/baseline/raw_reports/mfcc_integration.json</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:K12"/>
-  <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-</worksheet>
 </file>
</xml_diff>